<commit_message>
chore(examples): regenerate v2 examples with the implementation guide, cross-checks, survey context and round comparison
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: f9fd4a8a-033c-4218-b2f1-2c8da428242c
</commit_message>
<xml_diff>
--- a/referencia/exemplo-saida/pontuacao-v2-EXEMPLO.xlsx
+++ b/referencia/exemplo-saida/pontuacao-v2-EXEMPLO.xlsx
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Framework 2.0.1 · generated 2026-09-27</t>
+          <t>Framework 2.0.1 · generated 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4449,7 @@
         <v/>
       </c>
       <c r="E2">
-        <f>IF(D2="","",IF(D2&lt;0.8,"L0",IF(D2&lt;1.6,"L1",IF(D2&lt;2.4,"L2",IF(D2&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D2="","",IF(ROUND(D2,9)&lt;0.8,"L0",IF(ROUND(D2,9)&lt;1.6,"L1",IF(ROUND(D2,9)&lt;2.4,"L2",IF(ROUND(D2,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F2">
@@ -4485,7 +4485,7 @@
         <v/>
       </c>
       <c r="E3">
-        <f>IF(D3="","",IF(D3&lt;0.8,"L0",IF(D3&lt;1.6,"L1",IF(D3&lt;2.4,"L2",IF(D3&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D3="","",IF(ROUND(D3,9)&lt;0.8,"L0",IF(ROUND(D3,9)&lt;1.6,"L1",IF(ROUND(D3,9)&lt;2.4,"L2",IF(ROUND(D3,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F3">
@@ -4521,7 +4521,7 @@
         <v/>
       </c>
       <c r="E4">
-        <f>IF(D4="","",IF(D4&lt;0.8,"L0",IF(D4&lt;1.6,"L1",IF(D4&lt;2.4,"L2",IF(D4&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D4="","",IF(ROUND(D4,9)&lt;0.8,"L0",IF(ROUND(D4,9)&lt;1.6,"L1",IF(ROUND(D4,9)&lt;2.4,"L2",IF(ROUND(D4,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F4">
@@ -4557,7 +4557,7 @@
         <v/>
       </c>
       <c r="E5">
-        <f>IF(D5="","",IF(D5&lt;0.8,"L0",IF(D5&lt;1.6,"L1",IF(D5&lt;2.4,"L2",IF(D5&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D5="","",IF(ROUND(D5,9)&lt;0.8,"L0",IF(ROUND(D5,9)&lt;1.6,"L1",IF(ROUND(D5,9)&lt;2.4,"L2",IF(ROUND(D5,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F5">
@@ -4593,7 +4593,7 @@
         <v/>
       </c>
       <c r="E6">
-        <f>IF(D6="","",IF(D6&lt;0.8,"L0",IF(D6&lt;1.6,"L1",IF(D6&lt;2.4,"L2",IF(D6&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D6="","",IF(ROUND(D6,9)&lt;0.8,"L0",IF(ROUND(D6,9)&lt;1.6,"L1",IF(ROUND(D6,9)&lt;2.4,"L2",IF(ROUND(D6,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F6">
@@ -4629,7 +4629,7 @@
         <v/>
       </c>
       <c r="E7">
-        <f>IF(D7="","",IF(D7&lt;0.8,"L0",IF(D7&lt;1.6,"L1",IF(D7&lt;2.4,"L2",IF(D7&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D7="","",IF(ROUND(D7,9)&lt;0.8,"L0",IF(ROUND(D7,9)&lt;1.6,"L1",IF(ROUND(D7,9)&lt;2.4,"L2",IF(ROUND(D7,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F7">
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="E8">
-        <f>IF(D8="","",IF(D8&lt;0.8,"L0",IF(D8&lt;1.6,"L1",IF(D8&lt;2.4,"L2",IF(D8&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D8="","",IF(ROUND(D8,9)&lt;0.8,"L0",IF(ROUND(D8,9)&lt;1.6,"L1",IF(ROUND(D8,9)&lt;2.4,"L2",IF(ROUND(D8,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F8">
@@ -4701,7 +4701,7 @@
         <v/>
       </c>
       <c r="E9">
-        <f>IF(D9="","",IF(D9&lt;0.8,"L0",IF(D9&lt;1.6,"L1",IF(D9&lt;2.4,"L2",IF(D9&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D9="","",IF(ROUND(D9,9)&lt;0.8,"L0",IF(ROUND(D9,9)&lt;1.6,"L1",IF(ROUND(D9,9)&lt;2.4,"L2",IF(ROUND(D9,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F9">
@@ -4737,7 +4737,7 @@
         <v/>
       </c>
       <c r="E10">
-        <f>IF(D10="","",IF(D10&lt;0.8,"L0",IF(D10&lt;1.6,"L1",IF(D10&lt;2.4,"L2",IF(D10&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D10="","",IF(ROUND(D10,9)&lt;0.8,"L0",IF(ROUND(D10,9)&lt;1.6,"L1",IF(ROUND(D10,9)&lt;2.4,"L2",IF(ROUND(D10,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F10">
@@ -4773,7 +4773,7 @@
         <v/>
       </c>
       <c r="E11">
-        <f>IF(D11="","",IF(D11&lt;0.8,"L0",IF(D11&lt;1.6,"L1",IF(D11&lt;2.4,"L2",IF(D11&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D11="","",IF(ROUND(D11,9)&lt;0.8,"L0",IF(ROUND(D11,9)&lt;1.6,"L1",IF(ROUND(D11,9)&lt;2.4,"L2",IF(ROUND(D11,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F11">
@@ -4809,7 +4809,7 @@
         <v/>
       </c>
       <c r="E12">
-        <f>IF(D12="","",IF(D12&lt;0.8,"L0",IF(D12&lt;1.6,"L1",IF(D12&lt;2.4,"L2",IF(D12&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D12="","",IF(ROUND(D12,9)&lt;0.8,"L0",IF(ROUND(D12,9)&lt;1.6,"L1",IF(ROUND(D12,9)&lt;2.4,"L2",IF(ROUND(D12,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F12">
@@ -4845,7 +4845,7 @@
         <v/>
       </c>
       <c r="E13">
-        <f>IF(D13="","",IF(D13&lt;0.8,"L0",IF(D13&lt;1.6,"L1",IF(D13&lt;2.4,"L2",IF(D13&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D13="","",IF(ROUND(D13,9)&lt;0.8,"L0",IF(ROUND(D13,9)&lt;1.6,"L1",IF(ROUND(D13,9)&lt;2.4,"L2",IF(ROUND(D13,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F13">
@@ -4881,7 +4881,7 @@
         <v/>
       </c>
       <c r="E14">
-        <f>IF(D14="","",IF(D14&lt;0.8,"L0",IF(D14&lt;1.6,"L1",IF(D14&lt;2.4,"L2",IF(D14&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D14="","",IF(ROUND(D14,9)&lt;0.8,"L0",IF(ROUND(D14,9)&lt;1.6,"L1",IF(ROUND(D14,9)&lt;2.4,"L2",IF(ROUND(D14,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F14">
@@ -4917,7 +4917,7 @@
         <v/>
       </c>
       <c r="E15">
-        <f>IF(D15="","",IF(D15&lt;0.8,"L0",IF(D15&lt;1.6,"L1",IF(D15&lt;2.4,"L2",IF(D15&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D15="","",IF(ROUND(D15,9)&lt;0.8,"L0",IF(ROUND(D15,9)&lt;1.6,"L1",IF(ROUND(D15,9)&lt;2.4,"L2",IF(ROUND(D15,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F15">
@@ -4953,7 +4953,7 @@
         <v/>
       </c>
       <c r="E16">
-        <f>IF(D16="","",IF(D16&lt;0.8,"L0",IF(D16&lt;1.6,"L1",IF(D16&lt;2.4,"L2",IF(D16&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D16="","",IF(ROUND(D16,9)&lt;0.8,"L0",IF(ROUND(D16,9)&lt;1.6,"L1",IF(ROUND(D16,9)&lt;2.4,"L2",IF(ROUND(D16,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F16">
@@ -4989,7 +4989,7 @@
         <v/>
       </c>
       <c r="E17">
-        <f>IF(D17="","",IF(D17&lt;0.8,"L0",IF(D17&lt;1.6,"L1",IF(D17&lt;2.4,"L2",IF(D17&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D17="","",IF(ROUND(D17,9)&lt;0.8,"L0",IF(ROUND(D17,9)&lt;1.6,"L1",IF(ROUND(D17,9)&lt;2.4,"L2",IF(ROUND(D17,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F17">
@@ -5025,7 +5025,7 @@
         <v/>
       </c>
       <c r="E18">
-        <f>IF(D18="","",IF(D18&lt;0.8,"L0",IF(D18&lt;1.6,"L1",IF(D18&lt;2.4,"L2",IF(D18&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D18="","",IF(ROUND(D18,9)&lt;0.8,"L0",IF(ROUND(D18,9)&lt;1.6,"L1",IF(ROUND(D18,9)&lt;2.4,"L2",IF(ROUND(D18,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F18">
@@ -5061,7 +5061,7 @@
         <v/>
       </c>
       <c r="E19">
-        <f>IF(D19="","",IF(D19&lt;0.8,"L0",IF(D19&lt;1.6,"L1",IF(D19&lt;2.4,"L2",IF(D19&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D19="","",IF(ROUND(D19,9)&lt;0.8,"L0",IF(ROUND(D19,9)&lt;1.6,"L1",IF(ROUND(D19,9)&lt;2.4,"L2",IF(ROUND(D19,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F19">
@@ -5097,7 +5097,7 @@
         <v/>
       </c>
       <c r="E20">
-        <f>IF(D20="","",IF(D20&lt;0.8,"L0",IF(D20&lt;1.6,"L1",IF(D20&lt;2.4,"L2",IF(D20&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D20="","",IF(ROUND(D20,9)&lt;0.8,"L0",IF(ROUND(D20,9)&lt;1.6,"L1",IF(ROUND(D20,9)&lt;2.4,"L2",IF(ROUND(D20,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F20">
@@ -5133,7 +5133,7 @@
         <v/>
       </c>
       <c r="E21">
-        <f>IF(D21="","",IF(D21&lt;0.8,"L0",IF(D21&lt;1.6,"L1",IF(D21&lt;2.4,"L2",IF(D21&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D21="","",IF(ROUND(D21,9)&lt;0.8,"L0",IF(ROUND(D21,9)&lt;1.6,"L1",IF(ROUND(D21,9)&lt;2.4,"L2",IF(ROUND(D21,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F21">
@@ -5169,7 +5169,7 @@
         <v/>
       </c>
       <c r="E22">
-        <f>IF(D22="","",IF(D22&lt;0.8,"L0",IF(D22&lt;1.6,"L1",IF(D22&lt;2.4,"L2",IF(D22&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D22="","",IF(ROUND(D22,9)&lt;0.8,"L0",IF(ROUND(D22,9)&lt;1.6,"L1",IF(ROUND(D22,9)&lt;2.4,"L2",IF(ROUND(D22,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F22">
@@ -5205,7 +5205,7 @@
         <v/>
       </c>
       <c r="E23">
-        <f>IF(D23="","",IF(D23&lt;0.8,"L0",IF(D23&lt;1.6,"L1",IF(D23&lt;2.4,"L2",IF(D23&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D23="","",IF(ROUND(D23,9)&lt;0.8,"L0",IF(ROUND(D23,9)&lt;1.6,"L1",IF(ROUND(D23,9)&lt;2.4,"L2",IF(ROUND(D23,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F23">
@@ -5241,7 +5241,7 @@
         <v/>
       </c>
       <c r="E24">
-        <f>IF(D24="","",IF(D24&lt;0.8,"L0",IF(D24&lt;1.6,"L1",IF(D24&lt;2.4,"L2",IF(D24&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D24="","",IF(ROUND(D24,9)&lt;0.8,"L0",IF(ROUND(D24,9)&lt;1.6,"L1",IF(ROUND(D24,9)&lt;2.4,"L2",IF(ROUND(D24,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F24">
@@ -5277,7 +5277,7 @@
         <v/>
       </c>
       <c r="E25">
-        <f>IF(D25="","",IF(D25&lt;0.8,"L0",IF(D25&lt;1.6,"L1",IF(D25&lt;2.4,"L2",IF(D25&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D25="","",IF(ROUND(D25,9)&lt;0.8,"L0",IF(ROUND(D25,9)&lt;1.6,"L1",IF(ROUND(D25,9)&lt;2.4,"L2",IF(ROUND(D25,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F25">
@@ -5313,7 +5313,7 @@
         <v/>
       </c>
       <c r="E26">
-        <f>IF(D26="","",IF(D26&lt;0.8,"L0",IF(D26&lt;1.6,"L1",IF(D26&lt;2.4,"L2",IF(D26&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D26="","",IF(ROUND(D26,9)&lt;0.8,"L0",IF(ROUND(D26,9)&lt;1.6,"L1",IF(ROUND(D26,9)&lt;2.4,"L2",IF(ROUND(D26,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F26">
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="E27">
-        <f>IF(D27="","",IF(D27&lt;0.8,"L0",IF(D27&lt;1.6,"L1",IF(D27&lt;2.4,"L2",IF(D27&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D27="","",IF(ROUND(D27,9)&lt;0.8,"L0",IF(ROUND(D27,9)&lt;1.6,"L1",IF(ROUND(D27,9)&lt;2.4,"L2",IF(ROUND(D27,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F27">
@@ -5385,7 +5385,7 @@
         <v/>
       </c>
       <c r="E28">
-        <f>IF(D28="","",IF(D28&lt;0.8,"L0",IF(D28&lt;1.6,"L1",IF(D28&lt;2.4,"L2",IF(D28&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D28="","",IF(ROUND(D28,9)&lt;0.8,"L0",IF(ROUND(D28,9)&lt;1.6,"L1",IF(ROUND(D28,9)&lt;2.4,"L2",IF(ROUND(D28,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F28">
@@ -5421,7 +5421,7 @@
         <v/>
       </c>
       <c r="E29">
-        <f>IF(D29="","",IF(D29&lt;0.8,"L0",IF(D29&lt;1.6,"L1",IF(D29&lt;2.4,"L2",IF(D29&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D29="","",IF(ROUND(D29,9)&lt;0.8,"L0",IF(ROUND(D29,9)&lt;1.6,"L1",IF(ROUND(D29,9)&lt;2.4,"L2",IF(ROUND(D29,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F29">
@@ -5457,7 +5457,7 @@
         <v/>
       </c>
       <c r="E30">
-        <f>IF(D30="","",IF(D30&lt;0.8,"L0",IF(D30&lt;1.6,"L1",IF(D30&lt;2.4,"L2",IF(D30&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D30="","",IF(ROUND(D30,9)&lt;0.8,"L0",IF(ROUND(D30,9)&lt;1.6,"L1",IF(ROUND(D30,9)&lt;2.4,"L2",IF(ROUND(D30,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F30">
@@ -5493,7 +5493,7 @@
         <v/>
       </c>
       <c r="E31">
-        <f>IF(D31="","",IF(D31&lt;0.8,"L0",IF(D31&lt;1.6,"L1",IF(D31&lt;2.4,"L2",IF(D31&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D31="","",IF(ROUND(D31,9)&lt;0.8,"L0",IF(ROUND(D31,9)&lt;1.6,"L1",IF(ROUND(D31,9)&lt;2.4,"L2",IF(ROUND(D31,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F31">
@@ -5529,7 +5529,7 @@
         <v/>
       </c>
       <c r="E32">
-        <f>IF(D32="","",IF(D32&lt;0.8,"L0",IF(D32&lt;1.6,"L1",IF(D32&lt;2.4,"L2",IF(D32&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D32="","",IF(ROUND(D32,9)&lt;0.8,"L0",IF(ROUND(D32,9)&lt;1.6,"L1",IF(ROUND(D32,9)&lt;2.4,"L2",IF(ROUND(D32,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F32">
@@ -5565,7 +5565,7 @@
         <v/>
       </c>
       <c r="E33">
-        <f>IF(D33="","",IF(D33&lt;0.8,"L0",IF(D33&lt;1.6,"L1",IF(D33&lt;2.4,"L2",IF(D33&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D33="","",IF(ROUND(D33,9)&lt;0.8,"L0",IF(ROUND(D33,9)&lt;1.6,"L1",IF(ROUND(D33,9)&lt;2.4,"L2",IF(ROUND(D33,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F33">
@@ -5601,7 +5601,7 @@
         <v/>
       </c>
       <c r="E34">
-        <f>IF(D34="","",IF(D34&lt;0.8,"L0",IF(D34&lt;1.6,"L1",IF(D34&lt;2.4,"L2",IF(D34&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D34="","",IF(ROUND(D34,9)&lt;0.8,"L0",IF(ROUND(D34,9)&lt;1.6,"L1",IF(ROUND(D34,9)&lt;2.4,"L2",IF(ROUND(D34,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F34">
@@ -5637,7 +5637,7 @@
         <v/>
       </c>
       <c r="E35">
-        <f>IF(D35="","",IF(D35&lt;0.8,"L0",IF(D35&lt;1.6,"L1",IF(D35&lt;2.4,"L2",IF(D35&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D35="","",IF(ROUND(D35,9)&lt;0.8,"L0",IF(ROUND(D35,9)&lt;1.6,"L1",IF(ROUND(D35,9)&lt;2.4,"L2",IF(ROUND(D35,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F35">
@@ -5673,7 +5673,7 @@
         <v/>
       </c>
       <c r="E36">
-        <f>IF(D36="","",IF(D36&lt;0.8,"L0",IF(D36&lt;1.6,"L1",IF(D36&lt;2.4,"L2",IF(D36&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D36="","",IF(ROUND(D36,9)&lt;0.8,"L0",IF(ROUND(D36,9)&lt;1.6,"L1",IF(ROUND(D36,9)&lt;2.4,"L2",IF(ROUND(D36,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F36">
@@ -5709,7 +5709,7 @@
         <v/>
       </c>
       <c r="E37">
-        <f>IF(D37="","",IF(D37&lt;0.8,"L0",IF(D37&lt;1.6,"L1",IF(D37&lt;2.4,"L2",IF(D37&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D37="","",IF(ROUND(D37,9)&lt;0.8,"L0",IF(ROUND(D37,9)&lt;1.6,"L1",IF(ROUND(D37,9)&lt;2.4,"L2",IF(ROUND(D37,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F37">
@@ -5745,7 +5745,7 @@
         <v/>
       </c>
       <c r="E38">
-        <f>IF(D38="","",IF(D38&lt;0.8,"L0",IF(D38&lt;1.6,"L1",IF(D38&lt;2.4,"L2",IF(D38&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D38="","",IF(ROUND(D38,9)&lt;0.8,"L0",IF(ROUND(D38,9)&lt;1.6,"L1",IF(ROUND(D38,9)&lt;2.4,"L2",IF(ROUND(D38,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F38">
@@ -5781,7 +5781,7 @@
         <v/>
       </c>
       <c r="E39">
-        <f>IF(D39="","",IF(D39&lt;0.8,"L0",IF(D39&lt;1.6,"L1",IF(D39&lt;2.4,"L2",IF(D39&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D39="","",IF(ROUND(D39,9)&lt;0.8,"L0",IF(ROUND(D39,9)&lt;1.6,"L1",IF(ROUND(D39,9)&lt;2.4,"L2",IF(ROUND(D39,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F39">
@@ -5817,7 +5817,7 @@
         <v/>
       </c>
       <c r="E40">
-        <f>IF(D40="","",IF(D40&lt;0.8,"L0",IF(D40&lt;1.6,"L1",IF(D40&lt;2.4,"L2",IF(D40&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D40="","",IF(ROUND(D40,9)&lt;0.8,"L0",IF(ROUND(D40,9)&lt;1.6,"L1",IF(ROUND(D40,9)&lt;2.4,"L2",IF(ROUND(D40,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F40">
@@ -5853,7 +5853,7 @@
         <v/>
       </c>
       <c r="E41">
-        <f>IF(D41="","",IF(D41&lt;0.8,"L0",IF(D41&lt;1.6,"L1",IF(D41&lt;2.4,"L2",IF(D41&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D41="","",IF(ROUND(D41,9)&lt;0.8,"L0",IF(ROUND(D41,9)&lt;1.6,"L1",IF(ROUND(D41,9)&lt;2.4,"L2",IF(ROUND(D41,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F41">
@@ -5889,7 +5889,7 @@
         <v/>
       </c>
       <c r="E42">
-        <f>IF(D42="","",IF(D42&lt;0.8,"L0",IF(D42&lt;1.6,"L1",IF(D42&lt;2.4,"L2",IF(D42&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D42="","",IF(ROUND(D42,9)&lt;0.8,"L0",IF(ROUND(D42,9)&lt;1.6,"L1",IF(ROUND(D42,9)&lt;2.4,"L2",IF(ROUND(D42,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F42">
@@ -5925,7 +5925,7 @@
         <v/>
       </c>
       <c r="E43">
-        <f>IF(D43="","",IF(D43&lt;0.8,"L0",IF(D43&lt;1.6,"L1",IF(D43&lt;2.4,"L2",IF(D43&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D43="","",IF(ROUND(D43,9)&lt;0.8,"L0",IF(ROUND(D43,9)&lt;1.6,"L1",IF(ROUND(D43,9)&lt;2.4,"L2",IF(ROUND(D43,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F43">
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="E44">
-        <f>IF(D44="","",IF(D44&lt;0.8,"L0",IF(D44&lt;1.6,"L1",IF(D44&lt;2.4,"L2",IF(D44&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D44="","",IF(ROUND(D44,9)&lt;0.8,"L0",IF(ROUND(D44,9)&lt;1.6,"L1",IF(ROUND(D44,9)&lt;2.4,"L2",IF(ROUND(D44,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F44">
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="E45">
-        <f>IF(D45="","",IF(D45&lt;0.8,"L0",IF(D45&lt;1.6,"L1",IF(D45&lt;2.4,"L2",IF(D45&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D45="","",IF(ROUND(D45,9)&lt;0.8,"L0",IF(ROUND(D45,9)&lt;1.6,"L1",IF(ROUND(D45,9)&lt;2.4,"L2",IF(ROUND(D45,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F45">
@@ -6033,7 +6033,7 @@
         <v/>
       </c>
       <c r="E46">
-        <f>IF(D46="","",IF(D46&lt;0.8,"L0",IF(D46&lt;1.6,"L1",IF(D46&lt;2.4,"L2",IF(D46&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D46="","",IF(ROUND(D46,9)&lt;0.8,"L0",IF(ROUND(D46,9)&lt;1.6,"L1",IF(ROUND(D46,9)&lt;2.4,"L2",IF(ROUND(D46,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F46">
@@ -6069,7 +6069,7 @@
         <v/>
       </c>
       <c r="E47">
-        <f>IF(D47="","",IF(D47&lt;0.8,"L0",IF(D47&lt;1.6,"L1",IF(D47&lt;2.4,"L2",IF(D47&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D47="","",IF(ROUND(D47,9)&lt;0.8,"L0",IF(ROUND(D47,9)&lt;1.6,"L1",IF(ROUND(D47,9)&lt;2.4,"L2",IF(ROUND(D47,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F47">
@@ -6105,7 +6105,7 @@
         <v/>
       </c>
       <c r="E48">
-        <f>IF(D48="","",IF(D48&lt;0.8,"L0",IF(D48&lt;1.6,"L1",IF(D48&lt;2.4,"L2",IF(D48&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D48="","",IF(ROUND(D48,9)&lt;0.8,"L0",IF(ROUND(D48,9)&lt;1.6,"L1",IF(ROUND(D48,9)&lt;2.4,"L2",IF(ROUND(D48,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F48">
@@ -6141,7 +6141,7 @@
         <v/>
       </c>
       <c r="E49">
-        <f>IF(D49="","",IF(D49&lt;0.8,"L0",IF(D49&lt;1.6,"L1",IF(D49&lt;2.4,"L2",IF(D49&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D49="","",IF(ROUND(D49,9)&lt;0.8,"L0",IF(ROUND(D49,9)&lt;1.6,"L1",IF(ROUND(D49,9)&lt;2.4,"L2",IF(ROUND(D49,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F49">
@@ -6177,7 +6177,7 @@
         <v/>
       </c>
       <c r="E50">
-        <f>IF(D50="","",IF(D50&lt;0.8,"L0",IF(D50&lt;1.6,"L1",IF(D50&lt;2.4,"L2",IF(D50&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D50="","",IF(ROUND(D50,9)&lt;0.8,"L0",IF(ROUND(D50,9)&lt;1.6,"L1",IF(ROUND(D50,9)&lt;2.4,"L2",IF(ROUND(D50,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F50">
@@ -6213,7 +6213,7 @@
         <v/>
       </c>
       <c r="E51">
-        <f>IF(D51="","",IF(D51&lt;0.8,"L0",IF(D51&lt;1.6,"L1",IF(D51&lt;2.4,"L2",IF(D51&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D51="","",IF(ROUND(D51,9)&lt;0.8,"L0",IF(ROUND(D51,9)&lt;1.6,"L1",IF(ROUND(D51,9)&lt;2.4,"L2",IF(ROUND(D51,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F51">
@@ -6249,7 +6249,7 @@
         <v/>
       </c>
       <c r="E52">
-        <f>IF(D52="","",IF(D52&lt;0.8,"L0",IF(D52&lt;1.6,"L1",IF(D52&lt;2.4,"L2",IF(D52&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D52="","",IF(ROUND(D52,9)&lt;0.8,"L0",IF(ROUND(D52,9)&lt;1.6,"L1",IF(ROUND(D52,9)&lt;2.4,"L2",IF(ROUND(D52,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F52">
@@ -6285,7 +6285,7 @@
         <v/>
       </c>
       <c r="E53">
-        <f>IF(D53="","",IF(D53&lt;0.8,"L0",IF(D53&lt;1.6,"L1",IF(D53&lt;2.4,"L2",IF(D53&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D53="","",IF(ROUND(D53,9)&lt;0.8,"L0",IF(ROUND(D53,9)&lt;1.6,"L1",IF(ROUND(D53,9)&lt;2.4,"L2",IF(ROUND(D53,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F53">
@@ -6321,7 +6321,7 @@
         <v/>
       </c>
       <c r="E54">
-        <f>IF(D54="","",IF(D54&lt;0.8,"L0",IF(D54&lt;1.6,"L1",IF(D54&lt;2.4,"L2",IF(D54&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D54="","",IF(ROUND(D54,9)&lt;0.8,"L0",IF(ROUND(D54,9)&lt;1.6,"L1",IF(ROUND(D54,9)&lt;2.4,"L2",IF(ROUND(D54,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F54">
@@ -6357,7 +6357,7 @@
         <v/>
       </c>
       <c r="E55">
-        <f>IF(D55="","",IF(D55&lt;0.8,"L0",IF(D55&lt;1.6,"L1",IF(D55&lt;2.4,"L2",IF(D55&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D55="","",IF(ROUND(D55,9)&lt;0.8,"L0",IF(ROUND(D55,9)&lt;1.6,"L1",IF(ROUND(D55,9)&lt;2.4,"L2",IF(ROUND(D55,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F55">
@@ -6393,7 +6393,7 @@
         <v/>
       </c>
       <c r="E56">
-        <f>IF(D56="","",IF(D56&lt;0.8,"L0",IF(D56&lt;1.6,"L1",IF(D56&lt;2.4,"L2",IF(D56&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D56="","",IF(ROUND(D56,9)&lt;0.8,"L0",IF(ROUND(D56,9)&lt;1.6,"L1",IF(ROUND(D56,9)&lt;2.4,"L2",IF(ROUND(D56,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F56">
@@ -6429,7 +6429,7 @@
         <v/>
       </c>
       <c r="E57">
-        <f>IF(D57="","",IF(D57&lt;0.8,"L0",IF(D57&lt;1.6,"L1",IF(D57&lt;2.4,"L2",IF(D57&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D57="","",IF(ROUND(D57,9)&lt;0.8,"L0",IF(ROUND(D57,9)&lt;1.6,"L1",IF(ROUND(D57,9)&lt;2.4,"L2",IF(ROUND(D57,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F57">
@@ -6465,7 +6465,7 @@
         <v/>
       </c>
       <c r="E58">
-        <f>IF(D58="","",IF(D58&lt;0.8,"L0",IF(D58&lt;1.6,"L1",IF(D58&lt;2.4,"L2",IF(D58&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D58="","",IF(ROUND(D58,9)&lt;0.8,"L0",IF(ROUND(D58,9)&lt;1.6,"L1",IF(ROUND(D58,9)&lt;2.4,"L2",IF(ROUND(D58,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F58">
@@ -6501,7 +6501,7 @@
         <v/>
       </c>
       <c r="E59">
-        <f>IF(D59="","",IF(D59&lt;0.8,"L0",IF(D59&lt;1.6,"L1",IF(D59&lt;2.4,"L2",IF(D59&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D59="","",IF(ROUND(D59,9)&lt;0.8,"L0",IF(ROUND(D59,9)&lt;1.6,"L1",IF(ROUND(D59,9)&lt;2.4,"L2",IF(ROUND(D59,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F59">
@@ -6537,7 +6537,7 @@
         <v/>
       </c>
       <c r="E60">
-        <f>IF(D60="","",IF(D60&lt;0.8,"L0",IF(D60&lt;1.6,"L1",IF(D60&lt;2.4,"L2",IF(D60&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D60="","",IF(ROUND(D60,9)&lt;0.8,"L0",IF(ROUND(D60,9)&lt;1.6,"L1",IF(ROUND(D60,9)&lt;2.4,"L2",IF(ROUND(D60,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F60">
@@ -6573,7 +6573,7 @@
         <v/>
       </c>
       <c r="E61">
-        <f>IF(D61="","",IF(D61&lt;0.8,"L0",IF(D61&lt;1.6,"L1",IF(D61&lt;2.4,"L2",IF(D61&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D61="","",IF(ROUND(D61,9)&lt;0.8,"L0",IF(ROUND(D61,9)&lt;1.6,"L1",IF(ROUND(D61,9)&lt;2.4,"L2",IF(ROUND(D61,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F61">
@@ -6609,7 +6609,7 @@
         <v/>
       </c>
       <c r="E62">
-        <f>IF(D62="","",IF(D62&lt;0.8,"L0",IF(D62&lt;1.6,"L1",IF(D62&lt;2.4,"L2",IF(D62&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D62="","",IF(ROUND(D62,9)&lt;0.8,"L0",IF(ROUND(D62,9)&lt;1.6,"L1",IF(ROUND(D62,9)&lt;2.4,"L2",IF(ROUND(D62,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F62">
@@ -6723,7 +6723,7 @@
         <v/>
       </c>
       <c r="E2">
-        <f>IF(D2="","",IF(D2&lt;0.8,"L0",IF(D2&lt;1.6,"L1",IF(D2&lt;2.4,"L2",IF(D2&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D2="","",IF(ROUND(D2,9)&lt;0.8,"L0",IF(ROUND(D2,9)&lt;1.6,"L1",IF(ROUND(D2,9)&lt;2.4,"L2",IF(ROUND(D2,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F2" s="3" t="n">
@@ -6738,7 +6738,7 @@
         <v/>
       </c>
       <c r="I2">
-        <f>IF(H2="","",IF(H2&gt;=2.4,"P0",IF(H2&gt;=1.6,"P1",IF(H2&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H2="","",IF(ROUND(H2,9)&gt;=2.4,"P0",IF(ROUND(H2,9)&gt;=1.6,"P1",IF(ROUND(H2,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J2" s="3" t="n">
@@ -6772,7 +6772,7 @@
         <v/>
       </c>
       <c r="E3">
-        <f>IF(D3="","",IF(D3&lt;0.8,"L0",IF(D3&lt;1.6,"L1",IF(D3&lt;2.4,"L2",IF(D3&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D3="","",IF(ROUND(D3,9)&lt;0.8,"L0",IF(ROUND(D3,9)&lt;1.6,"L1",IF(ROUND(D3,9)&lt;2.4,"L2",IF(ROUND(D3,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F3" s="3" t="n">
@@ -6787,7 +6787,7 @@
         <v/>
       </c>
       <c r="I3">
-        <f>IF(H3="","",IF(H3&gt;=2.4,"P0",IF(H3&gt;=1.6,"P1",IF(H3&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H3="","",IF(ROUND(H3,9)&gt;=2.4,"P0",IF(ROUND(H3,9)&gt;=1.6,"P1",IF(ROUND(H3,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J3" s="3" t="n">
@@ -6821,7 +6821,7 @@
         <v/>
       </c>
       <c r="E4">
-        <f>IF(D4="","",IF(D4&lt;0.8,"L0",IF(D4&lt;1.6,"L1",IF(D4&lt;2.4,"L2",IF(D4&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D4="","",IF(ROUND(D4,9)&lt;0.8,"L0",IF(ROUND(D4,9)&lt;1.6,"L1",IF(ROUND(D4,9)&lt;2.4,"L2",IF(ROUND(D4,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F4" s="3" t="n">
@@ -6836,7 +6836,7 @@
         <v/>
       </c>
       <c r="I4">
-        <f>IF(H4="","",IF(H4&gt;=2.4,"P0",IF(H4&gt;=1.6,"P1",IF(H4&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H4="","",IF(ROUND(H4,9)&gt;=2.4,"P0",IF(ROUND(H4,9)&gt;=1.6,"P1",IF(ROUND(H4,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J4" s="3" t="n">
@@ -6859,7 +6859,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Code e engenharia de contexto</t>
+          <t>Código e engenharia de contexto</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -6870,7 +6870,7 @@
         <v/>
       </c>
       <c r="E5">
-        <f>IF(D5="","",IF(D5&lt;0.8,"L0",IF(D5&lt;1.6,"L1",IF(D5&lt;2.4,"L2",IF(D5&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D5="","",IF(ROUND(D5,9)&lt;0.8,"L0",IF(ROUND(D5,9)&lt;1.6,"L1",IF(ROUND(D5,9)&lt;2.4,"L2",IF(ROUND(D5,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F5" s="3" t="n">
@@ -6885,7 +6885,7 @@
         <v/>
       </c>
       <c r="I5">
-        <f>IF(H5="","",IF(H5&gt;=2.4,"P0",IF(H5&gt;=1.6,"P1",IF(H5&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H5="","",IF(ROUND(H5,9)&gt;=2.4,"P0",IF(ROUND(H5,9)&gt;=1.6,"P1",IF(ROUND(H5,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J5" s="3" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Review, qualidade e testes</t>
+          <t>Revisão, qualidade e testes</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -6919,7 +6919,7 @@
         <v/>
       </c>
       <c r="E6">
-        <f>IF(D6="","",IF(D6&lt;0.8,"L0",IF(D6&lt;1.6,"L1",IF(D6&lt;2.4,"L2",IF(D6&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D6="","",IF(ROUND(D6,9)&lt;0.8,"L0",IF(ROUND(D6,9)&lt;1.6,"L1",IF(ROUND(D6,9)&lt;2.4,"L2",IF(ROUND(D6,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F6" s="3" t="n">
@@ -6934,7 +6934,7 @@
         <v/>
       </c>
       <c r="I6">
-        <f>IF(H6="","",IF(H6&gt;=2.4,"P0",IF(H6&gt;=1.6,"P1",IF(H6&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H6="","",IF(ROUND(H6,9)&gt;=2.4,"P0",IF(ROUND(H6,9)&gt;=1.6,"P1",IF(ROUND(H6,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J6" s="3" t="n">
@@ -6957,7 +6957,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Segurança e AI Supply Chain</t>
+          <t>Segurança e cadeia de suprimentos de IA</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -6968,7 +6968,7 @@
         <v/>
       </c>
       <c r="E7">
-        <f>IF(D7="","",IF(D7&lt;0.8,"L0",IF(D7&lt;1.6,"L1",IF(D7&lt;2.4,"L2",IF(D7&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D7="","",IF(ROUND(D7,9)&lt;0.8,"L0",IF(ROUND(D7,9)&lt;1.6,"L1",IF(ROUND(D7,9)&lt;2.4,"L2",IF(ROUND(D7,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F7" s="3" t="n">
@@ -6983,7 +6983,7 @@
         <v/>
       </c>
       <c r="I7">
-        <f>IF(H7="","",IF(H7&gt;=2.4,"P0",IF(H7&gt;=1.6,"P1",IF(H7&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H7="","",IF(ROUND(H7,9)&gt;=2.4,"P0",IF(ROUND(H7,9)&gt;=1.6,"P1",IF(ROUND(H7,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J7" s="3" t="n">
@@ -7017,7 +7017,7 @@
         <v/>
       </c>
       <c r="E8">
-        <f>IF(D8="","",IF(D8&lt;0.8,"L0",IF(D8&lt;1.6,"L1",IF(D8&lt;2.4,"L2",IF(D8&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D8="","",IF(ROUND(D8,9)&lt;0.8,"L0",IF(ROUND(D8,9)&lt;1.6,"L1",IF(ROUND(D8,9)&lt;2.4,"L2",IF(ROUND(D8,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F8" s="3" t="n">
@@ -7032,7 +7032,7 @@
         <v/>
       </c>
       <c r="I8">
-        <f>IF(H8="","",IF(H8&gt;=2.4,"P0",IF(H8&gt;=1.6,"P1",IF(H8&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H8="","",IF(ROUND(H8,9)&gt;=2.4,"P0",IF(ROUND(H8,9)&gt;=1.6,"P1",IF(ROUND(H8,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J8" s="3" t="n">
@@ -7066,7 +7066,7 @@
         <v/>
       </c>
       <c r="E9">
-        <f>IF(D9="","",IF(D9&lt;0.8,"L0",IF(D9&lt;1.6,"L1",IF(D9&lt;2.4,"L2",IF(D9&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D9="","",IF(ROUND(D9,9)&lt;0.8,"L0",IF(ROUND(D9,9)&lt;1.6,"L1",IF(ROUND(D9,9)&lt;2.4,"L2",IF(ROUND(D9,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F9" s="3" t="n">
@@ -7081,7 +7081,7 @@
         <v/>
       </c>
       <c r="I9">
-        <f>IF(H9="","",IF(H9&gt;=2.4,"P0",IF(H9&gt;=1.6,"P1",IF(H9&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H9="","",IF(ROUND(H9,9)&gt;=2.4,"P0",IF(ROUND(H9,9)&gt;=1.6,"P1",IF(ROUND(H9,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J9" s="3" t="n">
@@ -7115,7 +7115,7 @@
         <v/>
       </c>
       <c r="E10">
-        <f>IF(D10="","",IF(D10&lt;0.8,"L0",IF(D10&lt;1.6,"L1",IF(D10&lt;2.4,"L2",IF(D10&lt;3.2,"L3","L4")))))</f>
+        <f>IF(D10="","",IF(ROUND(D10,9)&lt;0.8,"L0",IF(ROUND(D10,9)&lt;1.6,"L1",IF(ROUND(D10,9)&lt;2.4,"L2",IF(ROUND(D10,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="F10" s="3" t="n">
@@ -7130,7 +7130,7 @@
         <v/>
       </c>
       <c r="I10">
-        <f>IF(H10="","",IF(H10&gt;=2.4,"P0",IF(H10&gt;=1.6,"P1",IF(H10&gt;=0.9,"P2","P3"))))</f>
+        <f>IF(H10="","",IF(ROUND(H10,9)&gt;=2.4,"P0",IF(ROUND(H10,9)&gt;=1.6,"P1",IF(ROUND(H10,9)&gt;=0.9,"P2","P3"))))</f>
         <v/>
       </c>
       <c r="J10" s="3" t="n">
@@ -7202,7 +7202,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>IF(B2="","",IF(B2&lt;0.8,"L0",IF(B2&lt;1.6,"L1",IF(B2&lt;2.4,"L2",IF(B2&lt;3.2,"L3","L4")))))</f>
+        <f>IF(B2="","",IF(ROUND(B2,9)&lt;0.8,"L0",IF(ROUND(B2,9)&lt;1.6,"L1",IF(ROUND(B2,9)&lt;2.4,"L2",IF(ROUND(B2,9)&lt;3.2,"L3","L4")))))</f>
         <v/>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>